<commit_message>
Update negative price analysis 2026-08
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3440,6 +3440,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3451,7 +3485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6442,8 +6476,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B87">
+  <conditionalFormatting sqref="B2:B88">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6455,7 +6523,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C87">
+  <conditionalFormatting sqref="C2:C88">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6467,7 +6535,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D87">
+  <conditionalFormatting sqref="D2:D88">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6479,7 +6547,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E87">
+  <conditionalFormatting sqref="E2:E88">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6491,7 +6559,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F87">
+  <conditionalFormatting sqref="F2:F88">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6503,7 +6571,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G87">
+  <conditionalFormatting sqref="G2:G88">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6515,7 +6583,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H87">
+  <conditionalFormatting sqref="H2:H88">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6527,7 +6595,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I87">
+  <conditionalFormatting sqref="I2:I88">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6539,7 +6607,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J87">
+  <conditionalFormatting sqref="J2:J88">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6561,7 +6629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9816,6 +9884,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update negative price analysis 2026-09
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3474,6 +3474,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3485,7 +3519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6510,8 +6544,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B88">
+  <conditionalFormatting sqref="B2:B89">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6523,7 +6591,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C88">
+  <conditionalFormatting sqref="C2:C89">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6535,7 +6603,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D88">
+  <conditionalFormatting sqref="D2:D89">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6547,7 +6615,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E88">
+  <conditionalFormatting sqref="E2:E89">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6559,7 +6627,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F88">
+  <conditionalFormatting sqref="F2:F89">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6571,7 +6639,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G88">
+  <conditionalFormatting sqref="G2:G89">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6583,7 +6651,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H88">
+  <conditionalFormatting sqref="H2:H89">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6595,7 +6663,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I88">
+  <conditionalFormatting sqref="I2:I89">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6607,7 +6675,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J88">
+  <conditionalFormatting sqref="J2:J89">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6629,7 +6697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9921,6 +9989,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>